<commit_message>
feat: update excel templates formatting, strict data validation warnings and unlock action list sheet
</commit_message>
<xml_diff>
--- a/test-data/Master_Test_Suite.xlsx
+++ b/test-data/Master_Test_Suite.xlsx
@@ -1,24 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F4F58C-E111-4EFC-B25A-BEA640485964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2055" windowWidth="29040" windowHeight="15720" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-28920" yWindow="-2055" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="TEST_CASE" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="PAGE" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="ELEMENT" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="DATA_LOGIN" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="ACTION_LIST" state="visible" r:id="rId8"/>
+    <sheet name="TEST_CASE" sheetId="1" r:id="rId1"/>
+    <sheet name="PAGE" sheetId="2" r:id="rId2"/>
+    <sheet name="ELEMENT" sheetId="3" r:id="rId3"/>
+    <sheet name="DATA_LOGIN" sheetId="4" r:id="rId4"/>
+    <sheet name="ACTION_LIST" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="149">
   <si>
     <t>tc-id</t>
   </si>
@@ -71,16 +77,13 @@
     <t>url_sit_login</t>
   </si>
   <si>
-    <t>Error: page.goto: net::ERR_NAME_NOT_RESOLVED at https://sit-smh.vinmec.com/login</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>C:\Users\Admin\Documents\project\gui-testing-tool\reports\run_2026-05-19T17-37-29-925Z\screenshots\TC_LOGIN_001.png</t>
-  </si>
-  <si>
-    <t>0.36s</t>
+    <t>Navigated: url_sit_login</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>10.04s</t>
   </si>
   <si>
     <t>click</t>
@@ -89,6 +92,12 @@
     <t>btn_sit_login</t>
   </si>
   <si>
+    <t>Clicked on btn_sit_login</t>
+  </si>
+  <si>
+    <t>0.08s</t>
+  </si>
+  <si>
     <t>input</t>
   </si>
   <si>
@@ -98,21 +107,45 @@
     <t>$data_login.username</t>
   </si>
   <si>
+    <t>Input: 'admin@vinmec.com' into txt_username</t>
+  </si>
+  <si>
+    <t>0.99s</t>
+  </si>
+  <si>
     <t>txt_password</t>
   </si>
   <si>
     <t>$data_login.password</t>
   </si>
   <si>
+    <t>Input: 'Test@1234' into txt_password</t>
+  </si>
+  <si>
+    <t>0.04s</t>
+  </si>
+  <si>
     <t>btn_login</t>
   </si>
   <si>
+    <t>Clicked on btn_login</t>
+  </si>
+  <si>
+    <t>0.28s</t>
+  </si>
+  <si>
     <t>btn_dynamic_select</t>
   </si>
   <si>
     <t>$data_login.select_hospital</t>
   </si>
   <si>
+    <t>Clicked on btn_dynamic_select</t>
+  </si>
+  <si>
+    <t>1.00s</t>
+  </si>
+  <si>
     <t>check_status</t>
   </si>
   <si>
@@ -122,6 +155,15 @@
     <t>visible</t>
   </si>
   <si>
+    <t>Verified lbl_dashboard_data is visible</t>
+  </si>
+  <si>
+    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T05-25-48-354Z\screenshots\TC_LOGIN_001.png</t>
+  </si>
+  <si>
+    <t>0.06s</t>
+  </si>
+  <si>
     <t>TC_LOGIN_002</t>
   </si>
   <si>
@@ -131,13 +173,34 @@
     <t>neg</t>
   </si>
   <si>
-    <t>C:\Users\Admin\Documents\project\gui-testing-tool\reports\run_2026-05-19T17-37-29-925Z\screenshots\TC_LOGIN_002.png</t>
-  </si>
-  <si>
-    <t>0.17s</t>
+    <t>9.81s</t>
+  </si>
+  <si>
+    <t>0.07s</t>
+  </si>
+  <si>
+    <t>Input: 'admin@admin.com' into txt_username</t>
+  </si>
+  <si>
+    <t>0.95s</t>
+  </si>
+  <si>
+    <t>Input: 'admin123' into txt_password</t>
+  </si>
+  <si>
+    <t>0.19s</t>
   </si>
   <si>
     <t>error_msg</t>
+  </si>
+  <si>
+    <t>Verified error_msg is visible</t>
+  </si>
+  <si>
+    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T05-25-48-354Z\screenshots\TC_LOGIN_002.png</t>
+  </si>
+  <si>
+    <t>0.03s</t>
   </si>
   <si>
     <t>page</t>
@@ -413,27 +476,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
-      <family val="2"/>
-      <scheme val="minor"/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -442,23 +497,36 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <u/>
-      <color theme="10"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <name val="Consolas"/>
     </font>
   </fonts>
@@ -470,18 +538,18 @@
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A3A4A"/>
-        <bgColor rgb="001A3A4A"/>
+        <fgColor rgb="FF1A3A4A"/>
+        <bgColor rgb="FF1A3A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3F4F6"/>
-        <bgColor rgb="00F3F4F6"/>
+        <fgColor rgb="FFF3F4F6"/>
+        <bgColor rgb="FFF3F4F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -500,17 +568,25 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -566,12 +642,99 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -618,23 +781,12 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="00006100"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
-          <bgColor rgb="00C6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="009C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
-          <bgColor rgb="00FFC7CE"/>
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -651,34 +803,12 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="009C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
-          <bgColor rgb="00FFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="009C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
-          <bgColor rgb="00FFC7CE"/>
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1016,12 +1146,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L101"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.26953125" style="1" customWidth="1"/>
     <col min="2" max="2" width="40" style="1" customWidth="1"/>
@@ -1034,10 +1161,11 @@
     <col min="10" max="10" width="13.6328125" style="1" customWidth="1"/>
     <col min="11" max="11" width="13.7265625" style="1" customWidth="1"/>
     <col min="12" max="12" width="30" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.7265625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="8.7265625" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1075,7 +1203,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
@@ -1102,14 +1230,12 @@
       <c r="J2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="8"/>
+      <c r="L2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="5"/>
@@ -1117,19 +1243,25 @@
         <v>2</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>21</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>22</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="5"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
+      <c r="I3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-    </row>
-    <row r="4" ht="43.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L3" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="5"/>
@@ -1137,21 +1269,27 @@
         <v>3</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="5"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
+      <c r="I4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-    </row>
-    <row r="5" ht="29" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L4" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="5"/>
@@ -1159,21 +1297,27 @@
         <v>4</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H5" s="5"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
+      <c r="I5" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L5" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="5"/>
@@ -1181,19 +1325,25 @@
         <v>5</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="G6" s="7"/>
       <c r="H6" s="5"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
+      <c r="I6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-    </row>
-    <row r="7" ht="145" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L6" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="145" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="5"/>
@@ -1201,21 +1351,27 @@
         <v>6</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="I7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-    </row>
-    <row r="8" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="L7" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="145" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
@@ -1223,29 +1379,37 @@
         <v>7</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G8" s="9"/>
       <c r="H8" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D9" s="6">
         <v>1</v>
@@ -1264,14 +1428,12 @@
       <c r="J9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="8" t="s">
-        <v>37</v>
-      </c>
+      <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="5"/>
@@ -1279,19 +1441,25 @@
         <v>2</v>
       </c>
       <c r="E10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>21</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>22</v>
       </c>
       <c r="G10" s="9"/>
       <c r="H10" s="5"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
+      <c r="I10" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-    </row>
-    <row r="11" ht="29" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L10" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="5"/>
@@ -1299,21 +1467,27 @@
         <v>3</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H11" s="5"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="I11" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
-    </row>
-    <row r="12" ht="29" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L11" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="5"/>
@@ -1321,21 +1495,27 @@
         <v>4</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H12" s="5"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
+      <c r="I12" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-    </row>
-    <row r="13" ht="15.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L12" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
@@ -1343,19 +1523,25 @@
         <v>5</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="G13" s="9"/>
       <c r="H13" s="5"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
+      <c r="I13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
-    </row>
-    <row r="14" ht="145" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L13" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="145" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="5"/>
@@ -1363,21 +1549,29 @@
         <v>6</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="G14" s="9"/>
       <c r="H14" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="5"/>
@@ -1391,7 +1585,7 @@
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="5"/>
@@ -1405,7 +1599,7 @@
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="5"/>
@@ -1419,7 +1613,7 @@
       <c r="K17" s="8"/>
       <c r="L17" s="8"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="5"/>
@@ -1433,7 +1627,7 @@
       <c r="K18" s="8"/>
       <c r="L18" s="8"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="5"/>
@@ -1447,7 +1641,7 @@
       <c r="K19" s="8"/>
       <c r="L19" s="8"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="5"/>
@@ -1461,7 +1655,7 @@
       <c r="K20" s="8"/>
       <c r="L20" s="8"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="5"/>
@@ -1475,7 +1669,7 @@
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="5"/>
@@ -1489,7 +1683,7 @@
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="5"/>
@@ -1503,7 +1697,7 @@
       <c r="K23" s="8"/>
       <c r="L23" s="8"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="5"/>
@@ -1517,7 +1711,7 @@
       <c r="K24" s="8"/>
       <c r="L24" s="8"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="5"/>
@@ -1531,7 +1725,7 @@
       <c r="K25" s="8"/>
       <c r="L25" s="8"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="5"/>
@@ -1545,7 +1739,7 @@
       <c r="K26" s="8"/>
       <c r="L26" s="8"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="C27" s="5"/>
@@ -1559,7 +1753,7 @@
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="C28" s="5"/>
@@ -1573,7 +1767,7 @@
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="C29" s="5"/>
@@ -1587,7 +1781,7 @@
       <c r="K29" s="8"/>
       <c r="L29" s="8"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="C30" s="5"/>
@@ -1601,7 +1795,7 @@
       <c r="K30" s="8"/>
       <c r="L30" s="8"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="C31" s="5"/>
@@ -1615,7 +1809,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="C32" s="5"/>
@@ -1629,7 +1823,7 @@
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
       <c r="C33" s="5"/>
@@ -1643,7 +1837,7 @@
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="C34" s="5"/>
@@ -1657,7 +1851,7 @@
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="C35" s="5"/>
@@ -1671,7 +1865,7 @@
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="C36" s="5"/>
@@ -1685,7 +1879,7 @@
       <c r="K36" s="8"/>
       <c r="L36" s="8"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
       <c r="C37" s="5"/>
@@ -1699,7 +1893,7 @@
       <c r="K37" s="8"/>
       <c r="L37" s="8"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="C38" s="5"/>
@@ -1713,7 +1907,7 @@
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="C39" s="5"/>
@@ -1727,7 +1921,7 @@
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="C40" s="5"/>
@@ -1741,7 +1935,7 @@
       <c r="K40" s="8"/>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
       <c r="C41" s="5"/>
@@ -1755,7 +1949,7 @@
       <c r="K41" s="8"/>
       <c r="L41" s="8"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="C42" s="5"/>
@@ -1769,7 +1963,7 @@
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="5"/>
@@ -1783,7 +1977,7 @@
       <c r="K43" s="8"/>
       <c r="L43" s="8"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="C44" s="5"/>
@@ -1797,7 +1991,7 @@
       <c r="K44" s="8"/>
       <c r="L44" s="8"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="5"/>
@@ -1811,7 +2005,7 @@
       <c r="K45" s="8"/>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="5"/>
@@ -1825,7 +2019,7 @@
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="5"/>
@@ -1839,7 +2033,7 @@
       <c r="K47" s="8"/>
       <c r="L47" s="8"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="5"/>
@@ -1853,7 +2047,7 @@
       <c r="K48" s="8"/>
       <c r="L48" s="8"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="5"/>
@@ -1867,7 +2061,7 @@
       <c r="K49" s="8"/>
       <c r="L49" s="8"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="5"/>
@@ -1881,7 +2075,7 @@
       <c r="K50" s="8"/>
       <c r="L50" s="8"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" s="11"/>
       <c r="B51" s="4"/>
       <c r="C51" s="5"/>
@@ -1895,7 +2089,7 @@
       <c r="K51" s="12"/>
       <c r="L51" s="12"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" s="13"/>
       <c r="B52" s="13"/>
       <c r="C52" s="13"/>
@@ -1905,7 +2099,7 @@
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A53" s="13"/>
       <c r="B53" s="13"/>
       <c r="C53" s="13"/>
@@ -1915,7 +2109,7 @@
       <c r="G53" s="13"/>
       <c r="H53" s="13"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A54" s="13"/>
       <c r="B54" s="13"/>
       <c r="C54" s="13"/>
@@ -1925,7 +2119,7 @@
       <c r="G54" s="13"/>
       <c r="H54" s="13"/>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A55" s="13"/>
       <c r="B55" s="13"/>
       <c r="C55" s="13"/>
@@ -1935,7 +2129,7 @@
       <c r="G55" s="13"/>
       <c r="H55" s="13"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" s="13"/>
       <c r="B56" s="13"/>
       <c r="C56" s="13"/>
@@ -1945,7 +2139,7 @@
       <c r="G56" s="13"/>
       <c r="H56" s="13"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A57" s="13"/>
       <c r="B57" s="13"/>
       <c r="C57" s="13"/>
@@ -1955,7 +2149,7 @@
       <c r="G57" s="13"/>
       <c r="H57" s="13"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A58" s="13"/>
       <c r="B58" s="13"/>
       <c r="C58" s="13"/>
@@ -1965,7 +2159,7 @@
       <c r="G58" s="13"/>
       <c r="H58" s="13"/>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A59" s="13"/>
       <c r="B59" s="13"/>
       <c r="C59" s="13"/>
@@ -1975,7 +2169,7 @@
       <c r="G59" s="13"/>
       <c r="H59" s="13"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A60" s="13"/>
       <c r="B60" s="13"/>
       <c r="C60" s="13"/>
@@ -1985,7 +2179,7 @@
       <c r="G60" s="13"/>
       <c r="H60" s="13"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" s="13"/>
       <c r="B61" s="13"/>
       <c r="C61" s="13"/>
@@ -1995,7 +2189,7 @@
       <c r="G61" s="13"/>
       <c r="H61" s="13"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A62" s="13"/>
       <c r="B62" s="13"/>
       <c r="C62" s="13"/>
@@ -2005,7 +2199,7 @@
       <c r="G62" s="13"/>
       <c r="H62" s="13"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" s="13"/>
       <c r="B63" s="13"/>
       <c r="C63" s="13"/>
@@ -2015,7 +2209,7 @@
       <c r="G63" s="13"/>
       <c r="H63" s="13"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A64" s="13"/>
       <c r="B64" s="13"/>
       <c r="C64" s="13"/>
@@ -2025,7 +2219,7 @@
       <c r="G64" s="13"/>
       <c r="H64" s="13"/>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" s="13"/>
       <c r="B65" s="13"/>
       <c r="C65" s="13"/>
@@ -2035,7 +2229,7 @@
       <c r="G65" s="13"/>
       <c r="H65" s="13"/>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" s="13"/>
       <c r="B66" s="13"/>
       <c r="C66" s="13"/>
@@ -2045,7 +2239,7 @@
       <c r="G66" s="13"/>
       <c r="H66" s="13"/>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="13"/>
       <c r="B67" s="13"/>
       <c r="C67" s="13"/>
@@ -2055,7 +2249,7 @@
       <c r="G67" s="13"/>
       <c r="H67" s="13"/>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" s="13"/>
       <c r="B68" s="13"/>
       <c r="C68" s="13"/>
@@ -2065,7 +2259,7 @@
       <c r="G68" s="13"/>
       <c r="H68" s="13"/>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" s="13"/>
       <c r="B69" s="13"/>
       <c r="C69" s="13"/>
@@ -2075,7 +2269,7 @@
       <c r="G69" s="13"/>
       <c r="H69" s="13"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="13"/>
       <c r="B70" s="13"/>
       <c r="C70" s="13"/>
@@ -2085,7 +2279,7 @@
       <c r="G70" s="13"/>
       <c r="H70" s="13"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" s="13"/>
       <c r="B71" s="13"/>
       <c r="C71" s="13"/>
@@ -2095,7 +2289,7 @@
       <c r="G71" s="13"/>
       <c r="H71" s="13"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" s="13"/>
       <c r="B72" s="13"/>
       <c r="C72" s="13"/>
@@ -2105,7 +2299,7 @@
       <c r="G72" s="13"/>
       <c r="H72" s="13"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" s="13"/>
       <c r="B73" s="13"/>
       <c r="C73" s="13"/>
@@ -2115,7 +2309,7 @@
       <c r="G73" s="13"/>
       <c r="H73" s="13"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" s="13"/>
       <c r="B74" s="13"/>
       <c r="C74" s="13"/>
@@ -2125,7 +2319,7 @@
       <c r="G74" s="13"/>
       <c r="H74" s="13"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" s="13"/>
       <c r="B75" s="13"/>
       <c r="C75" s="13"/>
@@ -2135,7 +2329,7 @@
       <c r="G75" s="13"/>
       <c r="H75" s="13"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" s="13"/>
       <c r="B76" s="13"/>
       <c r="C76" s="13"/>
@@ -2145,7 +2339,7 @@
       <c r="G76" s="13"/>
       <c r="H76" s="13"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="13"/>
       <c r="B77" s="13"/>
       <c r="C77" s="13"/>
@@ -2155,7 +2349,7 @@
       <c r="G77" s="13"/>
       <c r="H77" s="13"/>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" s="13"/>
       <c r="B78" s="13"/>
       <c r="C78" s="13"/>
@@ -2165,7 +2359,7 @@
       <c r="G78" s="13"/>
       <c r="H78" s="13"/>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" s="13"/>
       <c r="B79" s="13"/>
       <c r="C79" s="13"/>
@@ -2175,7 +2369,7 @@
       <c r="G79" s="13"/>
       <c r="H79" s="13"/>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="13"/>
       <c r="B80" s="13"/>
       <c r="C80" s="13"/>
@@ -2185,7 +2379,7 @@
       <c r="G80" s="13"/>
       <c r="H80" s="13"/>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="13"/>
       <c r="B81" s="13"/>
       <c r="C81" s="13"/>
@@ -2195,7 +2389,7 @@
       <c r="G81" s="13"/>
       <c r="H81" s="13"/>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="13"/>
       <c r="B82" s="13"/>
       <c r="C82" s="13"/>
@@ -2205,7 +2399,7 @@
       <c r="G82" s="13"/>
       <c r="H82" s="13"/>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" s="13"/>
       <c r="B83" s="13"/>
       <c r="C83" s="13"/>
@@ -2215,7 +2409,7 @@
       <c r="G83" s="13"/>
       <c r="H83" s="13"/>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="13"/>
       <c r="B84" s="13"/>
       <c r="C84" s="13"/>
@@ -2225,7 +2419,7 @@
       <c r="G84" s="13"/>
       <c r="H84" s="13"/>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" s="13"/>
       <c r="B85" s="13"/>
       <c r="C85" s="13"/>
@@ -2235,7 +2429,7 @@
       <c r="G85" s="13"/>
       <c r="H85" s="13"/>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" s="13"/>
       <c r="B86" s="13"/>
       <c r="C86" s="13"/>
@@ -2245,7 +2439,7 @@
       <c r="G86" s="13"/>
       <c r="H86" s="13"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="13"/>
       <c r="B87" s="13"/>
       <c r="C87" s="13"/>
@@ -2255,7 +2449,7 @@
       <c r="G87" s="13"/>
       <c r="H87" s="13"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="13"/>
       <c r="B88" s="13"/>
       <c r="C88" s="13"/>
@@ -2265,7 +2459,7 @@
       <c r="G88" s="13"/>
       <c r="H88" s="13"/>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="13"/>
       <c r="B89" s="13"/>
       <c r="C89" s="13"/>
@@ -2275,7 +2469,7 @@
       <c r="G89" s="13"/>
       <c r="H89" s="13"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" s="13"/>
       <c r="B90" s="13"/>
       <c r="C90" s="13"/>
@@ -2285,7 +2479,7 @@
       <c r="G90" s="13"/>
       <c r="H90" s="13"/>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" s="13"/>
       <c r="B91" s="13"/>
       <c r="C91" s="13"/>
@@ -2295,7 +2489,7 @@
       <c r="G91" s="13"/>
       <c r="H91" s="13"/>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" s="13"/>
       <c r="B92" s="13"/>
       <c r="C92" s="13"/>
@@ -2305,7 +2499,7 @@
       <c r="G92" s="13"/>
       <c r="H92" s="13"/>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" s="13"/>
       <c r="B93" s="13"/>
       <c r="C93" s="13"/>
@@ -2315,7 +2509,7 @@
       <c r="G93" s="13"/>
       <c r="H93" s="13"/>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="13"/>
       <c r="B94" s="13"/>
       <c r="C94" s="13"/>
@@ -2325,7 +2519,7 @@
       <c r="G94" s="13"/>
       <c r="H94" s="13"/>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" s="13"/>
       <c r="B95" s="13"/>
       <c r="C95" s="13"/>
@@ -2335,7 +2529,7 @@
       <c r="G95" s="13"/>
       <c r="H95" s="13"/>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" s="13"/>
       <c r="B96" s="13"/>
       <c r="C96" s="13"/>
@@ -2345,7 +2539,7 @@
       <c r="G96" s="13"/>
       <c r="H96" s="13"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="13"/>
       <c r="B97" s="13"/>
       <c r="C97" s="13"/>
@@ -2355,7 +2549,7 @@
       <c r="G97" s="13"/>
       <c r="H97" s="13"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="13"/>
       <c r="B98" s="13"/>
       <c r="C98" s="13"/>
@@ -2365,7 +2559,7 @@
       <c r="G98" s="13"/>
       <c r="H98" s="13"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" s="13"/>
       <c r="B99" s="13"/>
       <c r="C99" s="13"/>
@@ -2375,7 +2569,7 @@
       <c r="G99" s="13"/>
       <c r="H99" s="13"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" s="13"/>
       <c r="B100" s="13"/>
       <c r="C100" s="13"/>
@@ -2385,7 +2579,7 @@
       <c r="G100" s="13"/>
       <c r="H100" s="13"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" s="13"/>
       <c r="B101" s="13"/>
       <c r="C101" s="13"/>
@@ -2398,315 +2592,324 @@
   </sheetData>
   <sheetProtection sheet="1" formatCells="0" insertRows="0" deleteRows="0"/>
   <conditionalFormatting sqref="J2:J7 J9:J101">
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="3" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J8">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J100">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="6" operator="equal">
+      <formula>"Failed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
+      <formula>"Passed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="C10:C100">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn 'pos' hoặc 'neg'." sqref="C2:C100" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"pos,neg"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C2:C100">
-      <formula1>"pos,neg"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E10:E100">
-      <formula1>OFFSET(ACTION_LIST!$A$2,0,0,COUNTA(ACTION_LIST!$A:$A)-1,1)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E2:E100">
-      <formula1>OFFSET(ACTION_LIST!$A$2,0,0,COUNTA(ACTION_LIST!$A:$A)-1,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng action từ danh sách ACTION_LIST." xr:uid="{00000000-0002-0000-0000-000002000000}">
+          <x14:formula1>
+            <xm:f>OFFSET(ACTION_LIST!$A$2,0,0,COUNTA(ACTION_LIST!$A:$A)-1,1)</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E100</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng target từ danh sách element_id của sheet ELEMENT." xr:uid="{00000000-0002-0000-0000-000004000000}">
+          <x14:formula1>
+            <xm:f>OFFSET(ELEMENT!$A$2,0,0,COUNTA(ELEMENT!$A:$A)-1,1)</xm:f>
+          </x14:formula1>
+          <xm:sqref>F2:F100</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.1796875" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" ht="15.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" ht="15.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A100">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>COUNTIF($A$2:$A$100,A2)&gt;1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>COUNTIF($A$2:$A$100,A2)&gt;1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>COUNTIF($A$2:$A$100,A2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1"/>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.453125" customWidth="1"/>
     <col min="2" max="2" width="11.26953125" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C5" s="16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="6" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>39</v>
-      </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" ht="14.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" ht="29" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A1000">
-    <cfRule type="expression" dxfId="8" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>COUNTIF($A$2:$A$1000,A2)&gt;1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>COUNTIF($A$2:$A$1000,A2)&gt;1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>COUNTIF($A$2:$A$1000,A2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="B10:B1000">
-      <formula1>"css,xpath,id,name,PAGE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B1000">
-      <formula1>"css,xpath,id,name,PAGE"</formula1>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng locator type từ danh sách." sqref="B2:B1000" xr:uid="{00000000-0002-0000-0200-000000000000}">
+      <formula1>"css,xpath,id,name,page"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:O10"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.36328125" customWidth="1"/>
     <col min="2" max="2" width="19.81640625" customWidth="1"/>
@@ -2714,18 +2917,18 @@
     <col min="4" max="4" width="40.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>54</v>
-      </c>
       <c r="D1" s="14" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="E1" s="14"/>
       <c r="F1" s="14"/>
@@ -2739,299 +2942,285 @@
       <c r="N1" s="14"/>
       <c r="O1" s="14"/>
     </row>
-    <row r="2" ht="15.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="17" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="17" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="4" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="A10:A100">
-      <formula1>"pos,neg"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="A2:A100">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn 'pos' hoặc 'neg'." sqref="A2:A100" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"pos,neg"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
-    <hyperlink ref="C2" r:id="rId2"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:B40"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+    <row r="1" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="16" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="4" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="8" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="9" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="10" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="11" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="12" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="B2" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="B13" s="16" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="20" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="14" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="16" t="s">
+      <c r="B3" s="21" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="15" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+    <row r="4" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B4" s="21" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="16" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+    <row r="5" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B5" s="21" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="17" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+    <row r="6" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B17" s="16" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="21" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="18" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="19" t="s">
+    <row r="8" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B8" s="21" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="19" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
+    <row r="9" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B9" s="21" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="20" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="19" t="s">
+    <row r="10" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B10" s="21" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="21" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+    <row r="11" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B11" s="21" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="22" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
+    <row r="12" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B12" s="21" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="23" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
+    <row r="13" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B13" s="21" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="24" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+    <row r="14" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B24" s="16" t="s">
+    </row>
+    <row r="15" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="20" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="25" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="19" t="s">
+      <c r="B15" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="B25" s="16" t="s">
+    </row>
+    <row r="16" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="20" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="26" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="19" t="s">
+      <c r="B16" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B26" s="16" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="20" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="27" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
+      <c r="B17" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="B27" s="16" t="s">
+    </row>
+    <row r="18" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="20" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="28" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="14.5" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B18" s="21" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="20"/>
+    </row>
+    <row r="29" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="20"/>
+    </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: optimize precondition logic, add relative paths for reports and build vaccination mock page
</commit_message>
<xml_diff>
--- a/test-data/Master_Test_Suite.xlsx
+++ b/test-data/Master_Test_Suite.xlsx
@@ -1,30 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F4F58C-E111-4EFC-B25A-BEA640485964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2055" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="TEST_CASE" sheetId="1" r:id="rId1"/>
-    <sheet name="PAGE" sheetId="2" r:id="rId2"/>
-    <sheet name="ELEMENT" sheetId="3" r:id="rId3"/>
-    <sheet name="DATA_LOGIN" sheetId="4" r:id="rId4"/>
-    <sheet name="ACTION_LIST" sheetId="5" r:id="rId5"/>
+    <sheet sheetId="1" name="TEST_CASE" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="PAGE" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="ELEMENT" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="DATA_LOGIN" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="ACTION_LIST" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="200">
   <si>
     <t>tc-id</t>
   </si>
@@ -83,7 +77,7 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>10.04s</t>
+    <t>2.99s</t>
   </si>
   <si>
     <t>click</t>
@@ -95,7 +89,7 @@
     <t>Clicked on btn_sit_login</t>
   </si>
   <si>
-    <t>0.08s</t>
+    <t>0.06s</t>
   </si>
   <si>
     <t>input</t>
@@ -110,7 +104,7 @@
     <t>Input: 'admin@vinmec.com' into txt_username</t>
   </si>
   <si>
-    <t>0.99s</t>
+    <t>0.93s</t>
   </si>
   <si>
     <t>txt_password</t>
@@ -131,7 +125,7 @@
     <t>Clicked on btn_login</t>
   </si>
   <si>
-    <t>0.28s</t>
+    <t>0.31s</t>
   </si>
   <si>
     <t>btn_dynamic_select</t>
@@ -143,7 +137,7 @@
     <t>Clicked on btn_dynamic_select</t>
   </si>
   <si>
-    <t>1.00s</t>
+    <t>1.38s</t>
   </si>
   <si>
     <t>check_status</t>
@@ -158,10 +152,10 @@
     <t>Verified lbl_dashboard_data is visible</t>
   </si>
   <si>
-    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T05-25-48-354Z\screenshots\TC_LOGIN_001.png</t>
-  </si>
-  <si>
-    <t>0.06s</t>
+    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T09-53-25-076Z\screenshots\TC_LOGIN_001.png</t>
+  </si>
+  <si>
+    <t>0.03s</t>
   </si>
   <si>
     <t>TC_LOGIN_002</t>
@@ -173,34 +167,151 @@
     <t>neg</t>
   </si>
   <si>
-    <t>9.81s</t>
-  </si>
-  <si>
-    <t>0.07s</t>
+    <t>3.63s</t>
   </si>
   <si>
     <t>Input: 'admin@admin.com' into txt_username</t>
   </si>
   <si>
-    <t>0.95s</t>
+    <t>0.91s</t>
   </si>
   <si>
     <t>Input: 'admin123' into txt_password</t>
   </si>
   <si>
+    <t>0.18s</t>
+  </si>
+  <si>
+    <t>error_msg</t>
+  </si>
+  <si>
+    <t>Verified error_msg is visible</t>
+  </si>
+  <si>
+    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T09-53-25-076Z\screenshots\TC_LOGIN_002.png</t>
+  </si>
+  <si>
+    <t>TC_VAC_001</t>
+  </si>
+  <si>
+    <t>Kiểm tra giao diện Dashboard Tiêm Chủng</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>call_tc</t>
+  </si>
+  <si>
+    <t>Called: TC_LOGIN_001</t>
+  </si>
+  <si>
+    <t>0.00s</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>url_vinmec_vaccine</t>
+  </si>
+  <si>
+    <t>Navigated: url_vinmec_vaccine</t>
+  </si>
+  <si>
+    <t>2.21s</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>lbl_card_cho_day_cdc</t>
+  </si>
+  <si>
+    <t>Verified lbl_card_cho_day_cdc is visible</t>
+  </si>
+  <si>
+    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T09-53-25-076Z\screenshots\TC_VAC_001.png</t>
+  </si>
+  <si>
+    <t>0.02s</t>
+  </si>
+  <si>
+    <t>TC_VAC_002</t>
+  </si>
+  <si>
+    <t>Kiểm tra chuyển hướng menu con 9.1.1 Điều phối tiêm chủng</t>
+  </si>
+  <si>
+    <t>Precondition 'TC_LOGIN_001' skipped (session active)</t>
+  </si>
+  <si>
+    <t>Refresh Precondition</t>
+  </si>
+  <si>
+    <t>Refreshed page</t>
+  </si>
+  <si>
+    <t>0.17s</t>
+  </si>
+  <si>
+    <t>2.20s</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>lnk_sidebar_dieupboi</t>
+  </si>
+  <si>
+    <t>Clicked on lnk_sidebar_dieupboi</t>
+  </si>
+  <si>
+    <t>0.09s</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>lbl_dieu_phoi_title</t>
+  </si>
+  <si>
+    <t>Verified lbl_dieu_phoi_title is visible</t>
+  </si>
+  <si>
+    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T09-53-25-076Z\screenshots\TC_VAC_002.png</t>
+  </si>
+  <si>
+    <t>0.23s</t>
+  </si>
+  <si>
+    <t>TC_VAC_003</t>
+  </si>
+  <si>
+    <t>Kiểm tra nút tương tác Xác nhận tiêm</t>
+  </si>
+  <si>
     <t>0.19s</t>
   </si>
   <si>
-    <t>error_msg</t>
-  </si>
-  <si>
-    <t>Verified error_msg is visible</t>
-  </si>
-  <si>
-    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T05-25-48-354Z\screenshots\TC_LOGIN_002.png</t>
-  </si>
-  <si>
-    <t>0.03s</t>
+    <t>2.18s</t>
+  </si>
+  <si>
+    <t>btn_xac_nhan_tiem</t>
+  </si>
+  <si>
+    <t>Clicked on btn_xac_nhan_tiem</t>
+  </si>
+  <si>
+    <t>lbl_modal_xac_nhan</t>
+  </si>
+  <si>
+    <t>Verified lbl_modal_xac_nhan is visible</t>
+  </si>
+  <si>
+    <t>C:\Users\datbt20\Documents\projects\gui-testing-tool\reports\run_2026-05-20T09-53-25-076Z\screenshots\TC_VAC_003.png</t>
+  </si>
+  <si>
+    <t>0.20s</t>
   </si>
   <si>
     <t>page</t>
@@ -224,6 +335,9 @@
     <t>https://sit-smh.vinmec.com/select-hospital</t>
   </si>
   <si>
+    <t>https://sit-smh.vinmec.com/vaccination</t>
+  </si>
+  <si>
     <t>element_id</t>
   </si>
   <si>
@@ -300,6 +414,39 @@
   </si>
   <si>
     <t>//span[text()='System Administrator']</t>
+  </si>
+  <si>
+    <t>menu_vaccination</t>
+  </si>
+  <si>
+    <t>//span[contains(text(), '9. Tiêm chủng')]</t>
+  </si>
+  <si>
+    <t>lbl_vaccination_dashboard_title</t>
+  </si>
+  <si>
+    <t>//*[contains(text(), 'Module 9')]</t>
+  </si>
+  <si>
+    <t>lbl_card_lich_tiem</t>
+  </si>
+  <si>
+    <t>(//*[contains(text(), 'Lịch tiêm hôm nay')])[1]</t>
+  </si>
+  <si>
+    <t>//*[contains(text(), 'Chờ đẩy CDC')]</t>
+  </si>
+  <si>
+    <t>//span[text()='9.1.1 Điều phối tiêm chủng']</t>
+  </si>
+  <si>
+    <t>//*[contains(text(), 'Chọn khách hàng ở cột trái')]</t>
+  </si>
+  <si>
+    <t>//button[contains(., 'Xác nhận tiêm')]</t>
+  </si>
+  <si>
+    <t>//h2[contains(text(), 'Xác nhận tiêm') or contains(text(), 'Thông tin tiêm')]</t>
   </si>
   <si>
     <t>test_case_type</t>
@@ -476,19 +623,27 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -497,36 +652,23 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <u/>
+      <color theme="10"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="12"/>
-      <color theme="10"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <name val="Consolas"/>
     </font>
   </fonts>
@@ -538,18 +680,18 @@
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A3A4A"/>
-        <bgColor rgb="FF1A3A4A"/>
+        <fgColor rgb="001A3A4A"/>
+        <bgColor rgb="001A3A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3F4F6"/>
-        <bgColor rgb="FFF3F4F6"/>
+        <fgColor rgb="00F3F4F6"/>
+        <bgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -568,18 +710,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -625,9 +759,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -657,7 +789,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -666,6 +809,50 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -693,122 +880,12 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="009C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1146,13 +1223,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L101"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:L100"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="21.26953125" style="1" customWidth="1"/>
     <col min="2" max="2" width="40" style="1" customWidth="1"/>
-    <col min="3" max="4" width="8.7265625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="25" style="1" customWidth="1"/>
     <col min="7" max="7" width="30" style="1" customWidth="1"/>
@@ -1161,11 +1242,10 @@
     <col min="10" max="10" width="13.6328125" style="1" customWidth="1"/>
     <col min="11" max="11" width="13.7265625" style="1" customWidth="1"/>
     <col min="12" max="12" width="30" style="1" customWidth="1"/>
-    <col min="13" max="13" width="8.7265625" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.7265625" style="1"/>
+    <col min="13" max="16384" width="8.7265625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1203,7 +1283,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
@@ -1235,7 +1315,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="5"/>
@@ -1261,7 +1341,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="5"/>
@@ -1289,7 +1369,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="5"/>
@@ -1317,7 +1397,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="5"/>
@@ -1343,7 +1423,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="145" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="5"/>
@@ -1371,7 +1451,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="145" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
@@ -1401,7 +1481,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>46</v>
       </c>
@@ -1433,7 +1513,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="5"/>
@@ -1456,10 +1536,10 @@
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="5"/>
@@ -1477,17 +1557,17 @@
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J11" s="8" t="s">
         <v>18</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="5"/>
@@ -1505,7 +1585,7 @@
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J12" s="8" t="s">
         <v>18</v>
@@ -1515,7 +1595,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" ht="15.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
@@ -1538,10 +1618,10 @@
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="145" customHeight="1" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="5"/>
@@ -1552,208 +1632,390 @@
         <v>40</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G14" s="9"/>
       <c r="H14" s="5" t="s">
         <v>42</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J14" s="8" t="s">
         <v>18</v>
       </c>
       <c r="K14" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="L14" s="8" t="s">
+      <c r="B15" s="4" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
+      <c r="C15" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>12</v>
+      </c>
       <c r="G15" s="7"/>
       <c r="H15" s="5"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
+      <c r="I15" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L15" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="5"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="10"/>
+      <c r="D16" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>64</v>
+      </c>
       <c r="G16" s="7"/>
       <c r="H16" s="5"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
+      <c r="I16" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L16" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="5"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
+      <c r="D17" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>68</v>
+      </c>
       <c r="G17" s="7"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
+      <c r="H17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>12</v>
+      </c>
       <c r="G18" s="7"/>
       <c r="H18" s="5"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+      <c r="I18" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L18" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="5"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="5"/>
+      <c r="D19" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>75</v>
+      </c>
       <c r="F19" s="5"/>
       <c r="G19" s="7"/>
       <c r="H19" s="5"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
+      <c r="I19" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L19" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="5"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
+      <c r="D20" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="G20" s="7"/>
       <c r="H20" s="5"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
+      <c r="I20" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L20" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="5"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
+      <c r="D21" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>80</v>
+      </c>
       <c r="G21" s="7"/>
       <c r="H21" s="5"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
+      <c r="I21" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L21" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="D22" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="G22" s="7"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
+      <c r="H22" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="L22" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>12</v>
+      </c>
       <c r="G23" s="7"/>
       <c r="H23" s="5"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="I23" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L23" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="5"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="5"/>
+      <c r="D24" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>75</v>
+      </c>
       <c r="F24" s="5"/>
       <c r="G24" s="7"/>
       <c r="H24" s="5"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
+      <c r="I24" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L24" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="5"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="D25" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="G25" s="7"/>
       <c r="H25" s="5"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
+      <c r="I25" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L25" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="5"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
+      <c r="D26" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>92</v>
+      </c>
       <c r="G26" s="7"/>
       <c r="H26" s="5"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
+      <c r="I26" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="K26" s="8"/>
-      <c r="L26" s="8"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L26" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="C27" s="5"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
+      <c r="D27" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="G27" s="7"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="H27" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="C28" s="5"/>
@@ -1767,7 +2029,7 @@
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="C29" s="5"/>
@@ -1781,7 +2043,7 @@
       <c r="K29" s="8"/>
       <c r="L29" s="8"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="C30" s="5"/>
@@ -1795,7 +2057,7 @@
       <c r="K30" s="8"/>
       <c r="L30" s="8"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="C31" s="5"/>
@@ -1809,7 +2071,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="C32" s="5"/>
@@ -1823,7 +2085,7 @@
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
       <c r="C33" s="5"/>
@@ -1837,7 +2099,7 @@
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="C34" s="5"/>
@@ -1851,7 +2113,7 @@
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="C35" s="5"/>
@@ -1865,7 +2127,7 @@
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="C36" s="5"/>
@@ -1879,7 +2141,7 @@
       <c r="K36" s="8"/>
       <c r="L36" s="8"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
       <c r="C37" s="5"/>
@@ -1893,7 +2155,7 @@
       <c r="K37" s="8"/>
       <c r="L37" s="8"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="C38" s="5"/>
@@ -1907,7 +2169,7 @@
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="C39" s="5"/>
@@ -1921,7 +2183,7 @@
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="C40" s="5"/>
@@ -1935,7 +2197,7 @@
       <c r="K40" s="8"/>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
       <c r="C41" s="5"/>
@@ -1949,7 +2211,7 @@
       <c r="K41" s="8"/>
       <c r="L41" s="8"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="C42" s="5"/>
@@ -1963,7 +2225,7 @@
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="5"/>
@@ -1977,7 +2239,7 @@
       <c r="K43" s="8"/>
       <c r="L43" s="8"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="C44" s="5"/>
@@ -1991,7 +2253,7 @@
       <c r="K44" s="8"/>
       <c r="L44" s="8"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="5"/>
@@ -2005,7 +2267,7 @@
       <c r="K45" s="8"/>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="5"/>
@@ -2019,7 +2281,7 @@
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="5"/>
@@ -2033,7 +2295,7 @@
       <c r="K47" s="8"/>
       <c r="L47" s="8"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="5"/>
@@ -2047,7 +2309,7 @@
       <c r="K48" s="8"/>
       <c r="L48" s="8"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="5"/>
@@ -2061,7 +2323,7 @@
       <c r="K49" s="8"/>
       <c r="L49" s="8"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="5"/>
@@ -2075,7 +2337,7 @@
       <c r="K50" s="8"/>
       <c r="L50" s="8"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="11"/>
       <c r="B51" s="4"/>
       <c r="C51" s="5"/>
@@ -2089,7 +2351,7 @@
       <c r="K51" s="12"/>
       <c r="L51" s="12"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="13"/>
       <c r="B52" s="13"/>
       <c r="C52" s="13"/>
@@ -2099,7 +2361,7 @@
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="13"/>
       <c r="B53" s="13"/>
       <c r="C53" s="13"/>
@@ -2109,7 +2371,7 @@
       <c r="G53" s="13"/>
       <c r="H53" s="13"/>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="13"/>
       <c r="B54" s="13"/>
       <c r="C54" s="13"/>
@@ -2119,7 +2381,7 @@
       <c r="G54" s="13"/>
       <c r="H54" s="13"/>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="13"/>
       <c r="B55" s="13"/>
       <c r="C55" s="13"/>
@@ -2129,7 +2391,7 @@
       <c r="G55" s="13"/>
       <c r="H55" s="13"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="13"/>
       <c r="B56" s="13"/>
       <c r="C56" s="13"/>
@@ -2139,7 +2401,7 @@
       <c r="G56" s="13"/>
       <c r="H56" s="13"/>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="13"/>
       <c r="B57" s="13"/>
       <c r="C57" s="13"/>
@@ -2149,7 +2411,7 @@
       <c r="G57" s="13"/>
       <c r="H57" s="13"/>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="13"/>
       <c r="B58" s="13"/>
       <c r="C58" s="13"/>
@@ -2159,7 +2421,7 @@
       <c r="G58" s="13"/>
       <c r="H58" s="13"/>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="13"/>
       <c r="B59" s="13"/>
       <c r="C59" s="13"/>
@@ -2169,7 +2431,7 @@
       <c r="G59" s="13"/>
       <c r="H59" s="13"/>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="13"/>
       <c r="B60" s="13"/>
       <c r="C60" s="13"/>
@@ -2179,7 +2441,7 @@
       <c r="G60" s="13"/>
       <c r="H60" s="13"/>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="13"/>
       <c r="B61" s="13"/>
       <c r="C61" s="13"/>
@@ -2189,7 +2451,7 @@
       <c r="G61" s="13"/>
       <c r="H61" s="13"/>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="13"/>
       <c r="B62" s="13"/>
       <c r="C62" s="13"/>
@@ -2199,7 +2461,7 @@
       <c r="G62" s="13"/>
       <c r="H62" s="13"/>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="13"/>
       <c r="B63" s="13"/>
       <c r="C63" s="13"/>
@@ -2209,7 +2471,7 @@
       <c r="G63" s="13"/>
       <c r="H63" s="13"/>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="13"/>
       <c r="B64" s="13"/>
       <c r="C64" s="13"/>
@@ -2219,7 +2481,7 @@
       <c r="G64" s="13"/>
       <c r="H64" s="13"/>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="13"/>
       <c r="B65" s="13"/>
       <c r="C65" s="13"/>
@@ -2229,7 +2491,7 @@
       <c r="G65" s="13"/>
       <c r="H65" s="13"/>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="13"/>
       <c r="B66" s="13"/>
       <c r="C66" s="13"/>
@@ -2239,7 +2501,7 @@
       <c r="G66" s="13"/>
       <c r="H66" s="13"/>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="13"/>
       <c r="B67" s="13"/>
       <c r="C67" s="13"/>
@@ -2249,7 +2511,7 @@
       <c r="G67" s="13"/>
       <c r="H67" s="13"/>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="13"/>
       <c r="B68" s="13"/>
       <c r="C68" s="13"/>
@@ -2259,7 +2521,7 @@
       <c r="G68" s="13"/>
       <c r="H68" s="13"/>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="13"/>
       <c r="B69" s="13"/>
       <c r="C69" s="13"/>
@@ -2269,7 +2531,7 @@
       <c r="G69" s="13"/>
       <c r="H69" s="13"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="13"/>
       <c r="B70" s="13"/>
       <c r="C70" s="13"/>
@@ -2279,7 +2541,7 @@
       <c r="G70" s="13"/>
       <c r="H70" s="13"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="13"/>
       <c r="B71" s="13"/>
       <c r="C71" s="13"/>
@@ -2289,7 +2551,7 @@
       <c r="G71" s="13"/>
       <c r="H71" s="13"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="13"/>
       <c r="B72" s="13"/>
       <c r="C72" s="13"/>
@@ -2299,7 +2561,7 @@
       <c r="G72" s="13"/>
       <c r="H72" s="13"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="13"/>
       <c r="B73" s="13"/>
       <c r="C73" s="13"/>
@@ -2309,7 +2571,7 @@
       <c r="G73" s="13"/>
       <c r="H73" s="13"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="13"/>
       <c r="B74" s="13"/>
       <c r="C74" s="13"/>
@@ -2319,7 +2581,7 @@
       <c r="G74" s="13"/>
       <c r="H74" s="13"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="13"/>
       <c r="B75" s="13"/>
       <c r="C75" s="13"/>
@@ -2329,7 +2591,7 @@
       <c r="G75" s="13"/>
       <c r="H75" s="13"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="13"/>
       <c r="B76" s="13"/>
       <c r="C76" s="13"/>
@@ -2339,7 +2601,7 @@
       <c r="G76" s="13"/>
       <c r="H76" s="13"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="13"/>
       <c r="B77" s="13"/>
       <c r="C77" s="13"/>
@@ -2349,7 +2611,7 @@
       <c r="G77" s="13"/>
       <c r="H77" s="13"/>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="13"/>
       <c r="B78" s="13"/>
       <c r="C78" s="13"/>
@@ -2359,7 +2621,7 @@
       <c r="G78" s="13"/>
       <c r="H78" s="13"/>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="13"/>
       <c r="B79" s="13"/>
       <c r="C79" s="13"/>
@@ -2369,7 +2631,7 @@
       <c r="G79" s="13"/>
       <c r="H79" s="13"/>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="13"/>
       <c r="B80" s="13"/>
       <c r="C80" s="13"/>
@@ -2379,7 +2641,7 @@
       <c r="G80" s="13"/>
       <c r="H80" s="13"/>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="13"/>
       <c r="B81" s="13"/>
       <c r="C81" s="13"/>
@@ -2389,7 +2651,7 @@
       <c r="G81" s="13"/>
       <c r="H81" s="13"/>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="13"/>
       <c r="B82" s="13"/>
       <c r="C82" s="13"/>
@@ -2399,7 +2661,7 @@
       <c r="G82" s="13"/>
       <c r="H82" s="13"/>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="13"/>
       <c r="B83" s="13"/>
       <c r="C83" s="13"/>
@@ -2409,7 +2671,7 @@
       <c r="G83" s="13"/>
       <c r="H83" s="13"/>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="13"/>
       <c r="B84" s="13"/>
       <c r="C84" s="13"/>
@@ -2419,7 +2681,7 @@
       <c r="G84" s="13"/>
       <c r="H84" s="13"/>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="13"/>
       <c r="B85" s="13"/>
       <c r="C85" s="13"/>
@@ -2429,7 +2691,7 @@
       <c r="G85" s="13"/>
       <c r="H85" s="13"/>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="13"/>
       <c r="B86" s="13"/>
       <c r="C86" s="13"/>
@@ -2439,7 +2701,7 @@
       <c r="G86" s="13"/>
       <c r="H86" s="13"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="13"/>
       <c r="B87" s="13"/>
       <c r="C87" s="13"/>
@@ -2449,7 +2711,7 @@
       <c r="G87" s="13"/>
       <c r="H87" s="13"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="13"/>
       <c r="B88" s="13"/>
       <c r="C88" s="13"/>
@@ -2459,7 +2721,7 @@
       <c r="G88" s="13"/>
       <c r="H88" s="13"/>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="13"/>
       <c r="B89" s="13"/>
       <c r="C89" s="13"/>
@@ -2469,7 +2731,7 @@
       <c r="G89" s="13"/>
       <c r="H89" s="13"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="13"/>
       <c r="B90" s="13"/>
       <c r="C90" s="13"/>
@@ -2479,7 +2741,7 @@
       <c r="G90" s="13"/>
       <c r="H90" s="13"/>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="13"/>
       <c r="B91" s="13"/>
       <c r="C91" s="13"/>
@@ -2489,7 +2751,7 @@
       <c r="G91" s="13"/>
       <c r="H91" s="13"/>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="13"/>
       <c r="B92" s="13"/>
       <c r="C92" s="13"/>
@@ -2499,7 +2761,7 @@
       <c r="G92" s="13"/>
       <c r="H92" s="13"/>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="13"/>
       <c r="B93" s="13"/>
       <c r="C93" s="13"/>
@@ -2509,7 +2771,7 @@
       <c r="G93" s="13"/>
       <c r="H93" s="13"/>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="13"/>
       <c r="B94" s="13"/>
       <c r="C94" s="13"/>
@@ -2519,7 +2781,7 @@
       <c r="G94" s="13"/>
       <c r="H94" s="13"/>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="13"/>
       <c r="B95" s="13"/>
       <c r="C95" s="13"/>
@@ -2529,7 +2791,7 @@
       <c r="G95" s="13"/>
       <c r="H95" s="13"/>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="13"/>
       <c r="B96" s="13"/>
       <c r="C96" s="13"/>
@@ -2539,7 +2801,7 @@
       <c r="G96" s="13"/>
       <c r="H96" s="13"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="13"/>
       <c r="B97" s="13"/>
       <c r="C97" s="13"/>
@@ -2549,7 +2811,7 @@
       <c r="G97" s="13"/>
       <c r="H97" s="13"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="13"/>
       <c r="B98" s="13"/>
       <c r="C98" s="13"/>
@@ -2559,7 +2821,7 @@
       <c r="G98" s="13"/>
       <c r="H98" s="13"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="13"/>
       <c r="B99" s="13"/>
       <c r="C99" s="13"/>
@@ -2569,7 +2831,7 @@
       <c r="G99" s="13"/>
       <c r="H99" s="13"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" s="13"/>
       <c r="B100" s="13"/>
       <c r="C100" s="13"/>
@@ -2578,338 +2840,421 @@
       <c r="F100" s="13"/>
       <c r="G100" s="13"/>
       <c r="H100" s="13"/>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A101" s="13"/>
-      <c r="B101" s="13"/>
-      <c r="C101" s="13"/>
-      <c r="D101" s="13"/>
-      <c r="E101" s="13"/>
-      <c r="F101" s="13"/>
-      <c r="G101" s="13"/>
-      <c r="H101" s="13"/>
+      <c r="L100" s="1"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" formatCells="0" insertRows="0" deleteRows="0"/>
-  <conditionalFormatting sqref="J2:J7 J9:J101">
-    <cfRule type="cellIs" dxfId="13" priority="3" operator="equal">
+  <conditionalFormatting sqref="J2:J51">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
-      <formula>"Failed"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J8">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
-      <formula>"Passed"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J100">
-    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="6" operator="equal">
-      <formula>"Failed"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
-      <formula>"Passed"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn 'pos' hoặc 'neg'." sqref="C2:C100" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn 'pos' hoặc 'neg'." sqref="C10:C100">
       <formula1>"pos,neg"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn 'pos' hoặc 'neg'." sqref="C2:C100">
+      <formula1>"pos,neg"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng action từ danh sách ACTION_LIST." sqref="E10:E100">
+      <formula1>OFFSET(ACTION_LIST!$A$2,0,0,COUNTA(ACTION_LIST!$A:$A)-1,1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng action từ danh sách ACTION_LIST." sqref="E2:E100">
+      <formula1>OFFSET(ACTION_LIST!$A$2,0,0,COUNTA(ACTION_LIST!$A:$A)-1,1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng target từ danh sách element_id của sheet ELEMENT." sqref="F10:F100">
+      <formula1>OFFSET(ELEMENT!$A$2,0,0,COUNTA(ELEMENT!$A:$A)-1,1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng target từ danh sách element_id của sheet ELEMENT." sqref="F2:F100">
+      <formula1>OFFSET(ELEMENT!$A$2,0,0,COUNTA(ELEMENT!$A:$A)-1,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng action từ danh sách ACTION_LIST." xr:uid="{00000000-0002-0000-0000-000002000000}">
-          <x14:formula1>
-            <xm:f>OFFSET(ACTION_LIST!$A$2,0,0,COUNTA(ACTION_LIST!$A:$A)-1,1)</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2:E100</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng target từ danh sách element_id của sheet ELEMENT." xr:uid="{00000000-0002-0000-0000-000004000000}">
-          <x14:formula1>
-            <xm:f>OFFSET(ELEMENT!$A$2,0,0,COUNTA(ELEMENT!$A:$A)-1,1)</xm:f>
-          </x14:formula1>
-          <xm:sqref>F2:F100</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="23.1796875" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" ht="15.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>59</v>
+        <v>98</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" ht="15.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>100</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" ht="15.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>65</v>
+      <c r="B5" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A100">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>COUNTIF($A$2:$A$100,A2)&gt;1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
-      <formula>COUNTIF($A$2:$A$100,A2)&gt;1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>COUNTIF($A$2:$A$100,A2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="B4" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20.453125" customWidth="1"/>
     <col min="2" max="2" width="11.26953125" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>66</v>
+        <v>106</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>67</v>
+        <v>107</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>109</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>109</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" ht="14.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>103</v>
       </c>
       <c r="B9" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" ht="29" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>109</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>85</v>
+        <v>125</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>109</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>127</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>41</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>91</v>
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>134</v>
+      </c>
+      <c r="B17" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" t="s">
+        <v>119</v>
+      </c>
+      <c r="C22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" t="s">
+        <v>119</v>
+      </c>
+      <c r="C23" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A1000">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>COUNTIF($A$2:$A$1000,A2)&gt;1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>COUNTIF($A$2:$A$1000,A2)&gt;1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+  <conditionalFormatting sqref="A2:A14 A16:A1000">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>COUNTIF($A$2:$A$1000,A2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng locator type từ danh sách." sqref="B2:B1000" xr:uid="{00000000-0002-0000-0200-000000000000}">
+  <conditionalFormatting sqref="A15">
+    <cfRule type="expression" dxfId="7" priority="1">
+      <formula>COUNTIF($A$2:$A$1000,A15)&gt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A1000">
+    <cfRule type="expression" dxfId="8" priority="3">
+      <formula>COUNTIF($A$2:$A$1000,A2)&gt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng locator type từ danh sách." sqref="B10:B1000">
+      <formula1>"css,xpath,id,name,page"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn đúng locator type từ danh sách." sqref="B2:B1000">
       <formula1>"css,xpath,id,name,page"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:O10"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="13.36328125" customWidth="1"/>
     <col min="2" max="2" width="19.81640625" customWidth="1"/>
@@ -2917,18 +3262,18 @@
     <col min="4" max="4" width="40.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" ht="15.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>92</v>
+        <v>143</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>72</v>
+        <v>112</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>73</v>
+        <v>113</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>93</v>
+        <v>144</v>
       </c>
       <c r="E1" s="14"/>
       <c r="F1" s="14"/>
@@ -2942,283 +3287,283 @@
       <c r="N1" s="14"/>
       <c r="O1" s="14"/>
     </row>
-    <row r="2" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="15.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>94</v>
+        <v>145</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>95</v>
+        <v>146</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>148</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="7" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="9" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="10" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="4" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn 'pos' hoặc 'neg'." sqref="A2:A100" xr:uid="{00000000-0002-0000-0300-000000000000}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn 'pos' hoặc 'neg'." sqref="A10:A100">
+      <formula1>"pos,neg"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Dữ liệu không hợp lệ" error="Vui lòng chọn 'pos' hoặc 'neg'." sqref="A2:A100">
       <formula1>"pos,neg"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
-    <hyperlink ref="C2" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="C2" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
-        <v>99</v>
+        <v>150</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>102</v>
+        <v>153</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
-        <v>104</v>
+        <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
-        <v>106</v>
+        <v>157</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
         <v>40</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
-        <v>110</v>
+        <v>161</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
-        <v>112</v>
+        <v>163</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
-        <v>114</v>
+        <v>165</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
-        <v>116</v>
+        <v>167</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
-        <v>118</v>
+        <v>169</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
-        <v>120</v>
+        <v>171</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
         <v>24</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="s">
-        <v>123</v>
+        <v>174</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
-        <v>125</v>
+        <v>176</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="20" t="s">
-        <v>127</v>
+        <v>178</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
-        <v>129</v>
+        <v>180</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
-        <v>131</v>
+        <v>182</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
-        <v>133</v>
+        <v>184</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
-        <v>135</v>
+        <v>186</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>137</v>
+        <v>188</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
-        <v>139</v>
+        <v>190</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
-        <v>141</v>
+        <v>192</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
-        <v>143</v>
+        <v>194</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
-        <v>145</v>
+        <v>196</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
-        <v>147</v>
+        <v>198</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="20"/>
-    </row>
-    <row r="29" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="20"/>
+        <v>199</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>